<commit_message>
Changes to the code of standardization
</commit_message>
<xml_diff>
--- a/cleaned_project_file.xlsx
+++ b/cleaned_project_file.xlsx
@@ -452,7 +452,7 @@
       <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Kansiime Theodora</t>
+          <t>Theodora Kansiime</t>
         </is>
       </c>
     </row>
@@ -470,7 +470,7 @@
       <c r="C3" t="inlineStr"/>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Hilda Oola</t>
+          <t>Oola Hilda</t>
         </is>
       </c>
     </row>
@@ -488,7 +488,7 @@
       <c r="C4" t="inlineStr"/>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Edward Esebu</t>
+          <t>Esebu Edward</t>
         </is>
       </c>
     </row>
@@ -506,7 +506,7 @@
       <c r="C5" t="inlineStr"/>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Norah Muwumba</t>
+          <t>Muwumba Norah</t>
         </is>
       </c>
     </row>
@@ -524,7 +524,7 @@
       <c r="C6" t="inlineStr"/>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Winfred Kababiito</t>
+          <t>Kababiito Winfred</t>
         </is>
       </c>
     </row>
@@ -542,7 +542,7 @@
       <c r="C7" t="inlineStr"/>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Naomi Tumuhimbise</t>
+          <t>Tumuhimbise Naomi</t>
         </is>
       </c>
     </row>
@@ -560,7 +560,7 @@
       <c r="C8" t="inlineStr"/>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Joanitah Namagembe</t>
+          <t>Namagembe Joanitah</t>
         </is>
       </c>
     </row>
@@ -578,7 +578,7 @@
       <c r="C9" t="inlineStr"/>
       <c r="D9" t="inlineStr">
         <is>
-          <t>James Kurawige</t>
+          <t>Kurawige James</t>
         </is>
       </c>
     </row>
@@ -596,7 +596,7 @@
       <c r="C10" t="inlineStr"/>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Edson Tumwesigye</t>
+          <t>Tumwesigye Edson</t>
         </is>
       </c>
     </row>
@@ -614,7 +614,7 @@
       <c r="C11" t="inlineStr"/>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Tito Lajja</t>
+          <t>Lajja Tito</t>
         </is>
       </c>
     </row>
@@ -632,7 +632,7 @@
       <c r="C12" t="inlineStr"/>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Arthur Kwarakunde</t>
+          <t>Kwarakunde Arthur</t>
         </is>
       </c>
     </row>
@@ -650,7 +650,7 @@
       <c r="C13" t="inlineStr"/>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Takia Nassozi</t>
+          <t>Nassozi Takia</t>
         </is>
       </c>
     </row>
@@ -668,7 +668,7 @@
       <c r="C14" t="inlineStr"/>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Joseline Kemigisha</t>
+          <t>Kemigisha Joseline</t>
         </is>
       </c>
     </row>
@@ -686,7 +686,7 @@
       <c r="C15" t="inlineStr"/>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Edith Kobusingye</t>
+          <t>Kobusingye Edith</t>
         </is>
       </c>
     </row>
@@ -704,7 +704,7 @@
       <c r="C16" t="inlineStr"/>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Geoffrey Kibwika</t>
+          <t>Kibwika Geoffrey</t>
         </is>
       </c>
     </row>
@@ -722,7 +722,7 @@
       <c r="C17" t="inlineStr"/>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Alice Akii-Bua</t>
+          <t>Akii-Bua Alice</t>
         </is>
       </c>
     </row>
@@ -740,7 +740,7 @@
       <c r="C18" t="inlineStr"/>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Noeline Muteesa</t>
+          <t>Muteesa Noeline</t>
         </is>
       </c>
     </row>
@@ -758,7 +758,7 @@
       <c r="C19" t="inlineStr"/>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Felix Langol</t>
+          <t>Langol Felix</t>
         </is>
       </c>
     </row>
@@ -776,7 +776,7 @@
       <c r="C20" t="inlineStr"/>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Donnah Kyakuwaire</t>
+          <t>Kyakuwaire Donnah</t>
         </is>
       </c>
     </row>
@@ -794,7 +794,7 @@
       <c r="C21" t="inlineStr"/>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Barbara Obonyo</t>
+          <t>Obonyo Barbara</t>
         </is>
       </c>
     </row>
@@ -812,7 +812,7 @@
       <c r="C22" t="inlineStr"/>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Godwin Madaraka</t>
+          <t>Madaraka Godwin</t>
         </is>
       </c>
     </row>
@@ -830,7 +830,7 @@
       <c r="C23" t="inlineStr"/>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Gift Andama</t>
+          <t>Andama Gift</t>
         </is>
       </c>
     </row>
@@ -848,7 +848,7 @@
       <c r="C24" t="inlineStr"/>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Evelyn Draru</t>
+          <t>Draru Evelyn</t>
         </is>
       </c>
     </row>
@@ -866,7 +866,7 @@
       <c r="C25" t="inlineStr"/>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Judith Kyarikunda</t>
+          <t>Kyarikunda Judith</t>
         </is>
       </c>
     </row>
@@ -884,7 +884,7 @@
       <c r="C26" t="inlineStr"/>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Paul Lifua</t>
+          <t>Lifua Paul</t>
         </is>
       </c>
     </row>
@@ -902,7 +902,7 @@
       <c r="C27" t="inlineStr"/>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Paula Oferu</t>
+          <t>Oferu Paula</t>
         </is>
       </c>
     </row>
@@ -920,7 +920,7 @@
       <c r="C28" t="inlineStr"/>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Ronald Jjuuko</t>
+          <t>Jjuuko Ronald</t>
         </is>
       </c>
     </row>
@@ -938,7 +938,7 @@
       <c r="C29" t="inlineStr"/>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Mugisha Mutifa</t>
+          <t>Mutifa Mugisha</t>
         </is>
       </c>
     </row>
@@ -956,7 +956,7 @@
       <c r="C30" t="inlineStr"/>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Jamada Isabirye</t>
+          <t>Isabirye Jamada</t>
         </is>
       </c>
     </row>
@@ -974,7 +974,7 @@
       <c r="C31" t="inlineStr"/>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Monica Nambi</t>
+          <t>Nambi Monica</t>
         </is>
       </c>
     </row>
@@ -992,7 +992,7 @@
       <c r="C32" t="inlineStr"/>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Jacqueline Uwera</t>
+          <t>Uwera Jacqueline</t>
         </is>
       </c>
     </row>
@@ -1010,7 +1010,7 @@
       <c r="C33" t="inlineStr"/>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Marion Ashaba-Aheebwa</t>
+          <t>Ashaba-Aheebwa Marion</t>
         </is>
       </c>
     </row>
@@ -1028,7 +1028,7 @@
       <c r="C34" t="inlineStr"/>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Miriam Kantono</t>
+          <t>Kantono Miriam</t>
         </is>
       </c>
     </row>
@@ -1046,7 +1046,7 @@
       <c r="C35" t="inlineStr"/>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Bogere Nalumansi</t>
+          <t>Nalumansi Bogere</t>
         </is>
       </c>
     </row>
@@ -1064,7 +1064,7 @@
       <c r="C36" t="inlineStr"/>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Robert Busuulwa</t>
+          <t>Busuulwa Robert</t>
         </is>
       </c>
     </row>
@@ -1082,7 +1082,7 @@
       <c r="C37" t="inlineStr"/>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Kassim Kasirye</t>
+          <t>Kasirye Kassim</t>
         </is>
       </c>
     </row>
@@ -1100,7 +1100,7 @@
       <c r="C38" t="inlineStr"/>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Joy Kansiime</t>
+          <t>Kansiime Joy</t>
         </is>
       </c>
     </row>
@@ -1118,7 +1118,7 @@
       <c r="C39" t="inlineStr"/>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Mudde Nabbona</t>
+          <t>Nabbona Mudde</t>
         </is>
       </c>
     </row>
@@ -1136,7 +1136,7 @@
       <c r="C40" t="inlineStr"/>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Elifazi Mutono</t>
+          <t>Mutono Elifazi</t>
         </is>
       </c>
     </row>
@@ -1154,7 +1154,7 @@
       <c r="C41" t="inlineStr"/>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Brian Otim</t>
+          <t>Otim Brian</t>
         </is>
       </c>
     </row>
@@ -1172,7 +1172,7 @@
       <c r="C42" t="inlineStr"/>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Proscovia Mbabazi</t>
+          <t>Mbabazi Proscovia</t>
         </is>
       </c>
     </row>
@@ -1190,7 +1190,7 @@
       <c r="C43" t="inlineStr"/>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Tayebwa Nyangoma</t>
+          <t>Nyangoma Tayebwa</t>
         </is>
       </c>
     </row>
@@ -1208,7 +1208,7 @@
       <c r="C44" t="inlineStr"/>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Doreen Busingye</t>
+          <t>Busingye Doreen</t>
         </is>
       </c>
     </row>
@@ -1226,7 +1226,7 @@
       <c r="C45" t="inlineStr"/>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Janan Munyambabazi</t>
+          <t>Munyambabazi Janan</t>
         </is>
       </c>
     </row>
@@ -1244,7 +1244,7 @@
       <c r="C46" t="inlineStr"/>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Brenda Aleesi</t>
+          <t>Aleesi Brenda</t>
         </is>
       </c>
     </row>
@@ -1262,7 +1262,7 @@
       <c r="C47" t="inlineStr"/>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Samson Woniaye</t>
+          <t>Woniaye Samson</t>
         </is>
       </c>
     </row>
@@ -1280,7 +1280,7 @@
       <c r="C48" t="inlineStr"/>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Christopher Kawenyera</t>
+          <t>Kawenyera Christopher</t>
         </is>
       </c>
     </row>
@@ -1298,7 +1298,7 @@
       <c r="C49" t="inlineStr"/>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Ivan Gwayambadde</t>
+          <t>Gwayambadde Ivan</t>
         </is>
       </c>
     </row>
@@ -1316,7 +1316,7 @@
       <c r="C50" t="inlineStr"/>
       <c r="D50" t="inlineStr">
         <is>
-          <t>Rose Nakimbugwe</t>
+          <t>Nakimbugwe Rose</t>
         </is>
       </c>
     </row>
@@ -1334,7 +1334,7 @@
       <c r="C51" t="inlineStr"/>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Julian Nankunda</t>
+          <t>Nankunda Julian</t>
         </is>
       </c>
     </row>
@@ -1352,7 +1352,7 @@
       <c r="C52" t="inlineStr"/>
       <c r="D52" t="inlineStr">
         <is>
-          <t>Winnie Kyomuhendo</t>
+          <t>Kyomuhendo Winnie</t>
         </is>
       </c>
     </row>
@@ -1370,7 +1370,7 @@
       <c r="C53" t="inlineStr"/>
       <c r="D53" t="inlineStr">
         <is>
-          <t>Ritah Ssonko</t>
+          <t>Ssonko Ritah</t>
         </is>
       </c>
     </row>
@@ -1388,7 +1388,7 @@
       <c r="C54" t="inlineStr"/>
       <c r="D54" t="inlineStr">
         <is>
-          <t>Henry Kirangwa</t>
+          <t>Kirangwa Henry</t>
         </is>
       </c>
     </row>
@@ -1406,7 +1406,7 @@
       <c r="C55" t="inlineStr"/>
       <c r="D55" t="inlineStr">
         <is>
-          <t>Eron Nangendo</t>
+          <t>Nangendo Eron</t>
         </is>
       </c>
     </row>
@@ -1424,7 +1424,7 @@
       <c r="C56" t="inlineStr"/>
       <c r="D56" t="inlineStr">
         <is>
-          <t>Isaac Mwebembezi</t>
+          <t>Mwebembezi Isaac</t>
         </is>
       </c>
     </row>
@@ -1442,7 +1442,7 @@
       <c r="C57" t="inlineStr"/>
       <c r="D57" t="inlineStr">
         <is>
-          <t>Charlotte Byarugaba</t>
+          <t>Byarugaba Charlotte</t>
         </is>
       </c>
     </row>
@@ -1460,7 +1460,7 @@
       <c r="C58" t="inlineStr"/>
       <c r="D58" t="inlineStr">
         <is>
-          <t>Yvonne Baranga</t>
+          <t>Baranga Yvonne</t>
         </is>
       </c>
     </row>
@@ -1478,7 +1478,7 @@
       <c r="C59" t="inlineStr"/>
       <c r="D59" t="inlineStr">
         <is>
-          <t>Farouq Vumya</t>
+          <t>Vumya Farouq</t>
         </is>
       </c>
     </row>
@@ -1496,7 +1496,7 @@
       <c r="C60" t="inlineStr"/>
       <c r="D60" t="inlineStr">
         <is>
-          <t>Brenda Mirembe</t>
+          <t>Mirembe Brenda</t>
         </is>
       </c>
     </row>
@@ -1514,7 +1514,7 @@
       <c r="C61" t="inlineStr"/>
       <c r="D61" t="inlineStr">
         <is>
-          <t>Sandra Magara</t>
+          <t>Magara Sandra</t>
         </is>
       </c>
     </row>
@@ -1532,7 +1532,7 @@
       <c r="C62" t="inlineStr"/>
       <c r="D62" t="inlineStr">
         <is>
-          <t>Gertrude Tibewanwa</t>
+          <t>Tibewanwa Gertrude</t>
         </is>
       </c>
     </row>
@@ -1550,7 +1550,7 @@
       <c r="C63" t="inlineStr"/>
       <c r="D63" t="inlineStr">
         <is>
-          <t>Phoebe Nantaba</t>
+          <t>Nantaba Phoebe</t>
         </is>
       </c>
     </row>
@@ -1568,7 +1568,7 @@
       <c r="C64" t="inlineStr"/>
       <c r="D64" t="inlineStr">
         <is>
-          <t>Luke Kayemba</t>
+          <t>Kayemba Luke</t>
         </is>
       </c>
     </row>
@@ -1586,7 +1586,7 @@
       <c r="C65" t="inlineStr"/>
       <c r="D65" t="inlineStr">
         <is>
-          <t>Agnes Birungi</t>
+          <t>Birungi Agnes</t>
         </is>
       </c>
     </row>
@@ -1604,7 +1604,7 @@
       <c r="C66" t="inlineStr"/>
       <c r="D66" t="inlineStr">
         <is>
-          <t>Murezi Ahumwire</t>
+          <t>Ahumwire Murezi</t>
         </is>
       </c>
     </row>
@@ -1622,7 +1622,7 @@
       <c r="C67" t="inlineStr"/>
       <c r="D67" t="inlineStr">
         <is>
-          <t>Ian Oyesigye</t>
+          <t>Oyesigye Ian</t>
         </is>
       </c>
     </row>
@@ -1640,7 +1640,7 @@
       <c r="C68" t="inlineStr"/>
       <c r="D68" t="inlineStr">
         <is>
-          <t>Javan Muhangi</t>
+          <t>Muhangi Javan</t>
         </is>
       </c>
     </row>
@@ -1658,7 +1658,7 @@
       <c r="C69" t="inlineStr"/>
       <c r="D69" t="inlineStr">
         <is>
-          <t>Arnold Mpairwe</t>
+          <t>Mpairwe Arnold</t>
         </is>
       </c>
     </row>
@@ -1676,7 +1676,7 @@
       <c r="C70" t="inlineStr"/>
       <c r="D70" t="inlineStr">
         <is>
-          <t>Ivan Twehamye</t>
+          <t>Twehamye Ivan</t>
         </is>
       </c>
     </row>
@@ -1694,7 +1694,7 @@
       <c r="C71" t="inlineStr"/>
       <c r="D71" t="inlineStr">
         <is>
-          <t>Fortunate Rukundo</t>
+          <t>Rukundo Fortunate</t>
         </is>
       </c>
     </row>
@@ -1712,7 +1712,7 @@
       <c r="C72" t="inlineStr"/>
       <c r="D72" t="inlineStr">
         <is>
-          <t>Arthur Ngasirwa</t>
+          <t>Ngasirwa Arthur</t>
         </is>
       </c>
     </row>
@@ -1730,7 +1730,7 @@
       <c r="C73" t="inlineStr"/>
       <c r="D73" t="inlineStr">
         <is>
-          <t>Violet Najjingo</t>
+          <t>Najjingo Violet</t>
         </is>
       </c>
     </row>
@@ -1748,7 +1748,7 @@
       <c r="C74" t="inlineStr"/>
       <c r="D74" t="inlineStr">
         <is>
-          <t>Vivian Nabbosa</t>
+          <t>Nabbosa Vivian</t>
         </is>
       </c>
     </row>
@@ -1766,7 +1766,7 @@
       <c r="C75" t="inlineStr"/>
       <c r="D75" t="inlineStr">
         <is>
-          <t>Paul Kiiza</t>
+          <t>Kiiza Paul</t>
         </is>
       </c>
     </row>
@@ -1784,7 +1784,7 @@
       <c r="C76" t="inlineStr"/>
       <c r="D76" t="inlineStr">
         <is>
-          <t>Kizito Kanyike</t>
+          <t>Kanyike Kizito</t>
         </is>
       </c>
     </row>
@@ -1802,7 +1802,7 @@
       <c r="C77" t="inlineStr"/>
       <c r="D77" t="inlineStr">
         <is>
-          <t>Moses Kwanya</t>
+          <t>Kwanya Moses</t>
         </is>
       </c>
     </row>
@@ -1820,7 +1820,7 @@
       <c r="C78" t="inlineStr"/>
       <c r="D78" t="inlineStr">
         <is>
-          <t>Collins Bangirana</t>
+          <t>Bangirana Collins</t>
         </is>
       </c>
     </row>
@@ -1838,7 +1838,7 @@
       <c r="C79" t="inlineStr"/>
       <c r="D79" t="inlineStr">
         <is>
-          <t>Ignatius Mawanda</t>
+          <t>Mawanda Ignatius</t>
         </is>
       </c>
     </row>
@@ -1856,7 +1856,7 @@
       <c r="C80" t="inlineStr"/>
       <c r="D80" t="inlineStr">
         <is>
-          <t>Kenneth Karara</t>
+          <t>Karara Kenneth</t>
         </is>
       </c>
     </row>
@@ -1874,7 +1874,7 @@
       <c r="C81" t="inlineStr"/>
       <c r="D81" t="inlineStr">
         <is>
-          <t>Diana Akurut</t>
+          <t>Akurut Diana</t>
         </is>
       </c>
     </row>
@@ -1892,7 +1892,7 @@
       <c r="C82" t="inlineStr"/>
       <c r="D82" t="inlineStr">
         <is>
-          <t>Eunice Ayebazibwe</t>
+          <t>Ayebazibwe Eunice</t>
         </is>
       </c>
     </row>
@@ -1910,7 +1910,7 @@
       <c r="C83" t="inlineStr"/>
       <c r="D83" t="inlineStr">
         <is>
-          <t>Frances Nakabuye</t>
+          <t>Nakabuye Frances</t>
         </is>
       </c>
     </row>
@@ -1928,7 +1928,7 @@
       <c r="C84" t="inlineStr"/>
       <c r="D84" t="inlineStr">
         <is>
-          <t>Martin Wagabaza</t>
+          <t>Wagabaza Martin</t>
         </is>
       </c>
     </row>
@@ -1946,7 +1946,7 @@
       <c r="C85" t="inlineStr"/>
       <c r="D85" t="inlineStr">
         <is>
-          <t>Alex Arinda</t>
+          <t>Arinda Alex</t>
         </is>
       </c>
     </row>
@@ -1964,7 +1964,7 @@
       <c r="C86" t="inlineStr"/>
       <c r="D86" t="inlineStr">
         <is>
-          <t>Uthman Kirunda</t>
+          <t>Kirunda Uthman</t>
         </is>
       </c>
     </row>
@@ -1982,7 +1982,7 @@
       <c r="C87" t="inlineStr"/>
       <c r="D87" t="inlineStr">
         <is>
-          <t>Dancan Taremwa</t>
+          <t>Taremwa Dancan</t>
         </is>
       </c>
     </row>
@@ -2000,7 +2000,7 @@
       <c r="C88" t="inlineStr"/>
       <c r="D88" t="inlineStr">
         <is>
-          <t>Olivia Vivianah Atuheire</t>
+          <t>Atuheire Vivianah</t>
         </is>
       </c>
     </row>
@@ -2018,7 +2018,7 @@
       <c r="C89" t="inlineStr"/>
       <c r="D89" t="inlineStr">
         <is>
-          <t>Barole Mugume</t>
+          <t>Mugume Barole</t>
         </is>
       </c>
     </row>
@@ -2036,7 +2036,7 @@
       <c r="C90" t="inlineStr"/>
       <c r="D90" t="inlineStr">
         <is>
-          <t>Ruth Rebecca Kauma</t>
+          <t>Kauma Rebecca</t>
         </is>
       </c>
     </row>
@@ -2054,7 +2054,7 @@
       <c r="C91" t="inlineStr"/>
       <c r="D91" t="inlineStr">
         <is>
-          <t>Ndagire Mable</t>
+          <t>Mable Ndagire</t>
         </is>
       </c>
     </row>
@@ -2072,7 +2072,7 @@
       <c r="C92" t="inlineStr"/>
       <c r="D92" t="inlineStr">
         <is>
-          <t>James Warugaba</t>
+          <t>Warugaba James</t>
         </is>
       </c>
     </row>
@@ -2090,7 +2090,7 @@
       <c r="C93" t="inlineStr"/>
       <c r="D93" t="inlineStr">
         <is>
-          <t>William Kasangaki</t>
+          <t>Kasangaki William</t>
         </is>
       </c>
     </row>
@@ -2108,7 +2108,7 @@
       <c r="C94" t="inlineStr"/>
       <c r="D94" t="inlineStr">
         <is>
-          <t>Hafuswa Nakitende</t>
+          <t>Nakitende Hafuswa</t>
         </is>
       </c>
     </row>
@@ -2126,7 +2126,7 @@
       <c r="C95" t="inlineStr"/>
       <c r="D95" t="inlineStr">
         <is>
-          <t>Dennis Wabwire</t>
+          <t>Wabwire Dennis</t>
         </is>
       </c>
     </row>
@@ -2144,7 +2144,7 @@
       <c r="C96" t="inlineStr"/>
       <c r="D96" t="inlineStr">
         <is>
-          <t>Ruth Totto</t>
+          <t>Totto Ruth</t>
         </is>
       </c>
     </row>
@@ -2162,7 +2162,7 @@
       <c r="C97" t="inlineStr"/>
       <c r="D97" t="inlineStr">
         <is>
-          <t>Andrew Kayongo</t>
+          <t>Kayongo Andrew</t>
         </is>
       </c>
     </row>
@@ -2180,7 +2180,7 @@
       <c r="C98" t="inlineStr"/>
       <c r="D98" t="inlineStr">
         <is>
-          <t>Poover Kyomugisha</t>
+          <t>Kyomugisha Poover</t>
         </is>
       </c>
     </row>
@@ -2198,7 +2198,7 @@
       <c r="C99" t="inlineStr"/>
       <c r="D99" t="inlineStr">
         <is>
-          <t>Priscilla Awino</t>
+          <t>Awino Priscilla</t>
         </is>
       </c>
     </row>
@@ -2216,7 +2216,7 @@
       <c r="C100" t="inlineStr"/>
       <c r="D100" t="inlineStr">
         <is>
-          <t>Teddy Nabacwa</t>
+          <t>Nabacwa Teddy</t>
         </is>
       </c>
     </row>
@@ -2234,7 +2234,7 @@
       <c r="C101" t="inlineStr"/>
       <c r="D101" t="inlineStr">
         <is>
-          <t>Aisha Nandawula</t>
+          <t>Nandawula Aisha</t>
         </is>
       </c>
     </row>
@@ -2252,7 +2252,7 @@
       <c r="C102" t="inlineStr"/>
       <c r="D102" t="inlineStr">
         <is>
-          <t>Sandra Amongi</t>
+          <t>Amongi Sandra</t>
         </is>
       </c>
     </row>
@@ -2270,7 +2270,7 @@
       <c r="C103" t="inlineStr"/>
       <c r="D103" t="inlineStr">
         <is>
-          <t>Francis Kaweesi</t>
+          <t>Kaweesi Francis</t>
         </is>
       </c>
     </row>
@@ -2288,7 +2288,7 @@
       <c r="C104" t="inlineStr"/>
       <c r="D104" t="inlineStr">
         <is>
-          <t>Jackson Kobwemi</t>
+          <t>Kobwemi Jackson</t>
         </is>
       </c>
     </row>
@@ -2306,7 +2306,7 @@
       <c r="C105" t="inlineStr"/>
       <c r="D105" t="inlineStr">
         <is>
-          <t>Godfrey Tumwine</t>
+          <t>Tumwine Godfrey</t>
         </is>
       </c>
     </row>
@@ -2324,7 +2324,7 @@
       <c r="C106" t="inlineStr"/>
       <c r="D106" t="inlineStr">
         <is>
-          <t>Fednandi Ariho</t>
+          <t>Ariho Fednandi</t>
         </is>
       </c>
     </row>
@@ -2342,7 +2342,7 @@
       <c r="C107" t="inlineStr"/>
       <c r="D107" t="inlineStr">
         <is>
-          <t>Kyarukunda Sharon</t>
+          <t>Sharon Kyarukunda</t>
         </is>
       </c>
     </row>
@@ -2360,7 +2360,7 @@
       <c r="C108" t="inlineStr"/>
       <c r="D108" t="inlineStr">
         <is>
-          <t>Babwetera Jolly</t>
+          <t>Jolly Babwetera</t>
         </is>
       </c>
     </row>
@@ -2378,7 +2378,7 @@
       <c r="C109" t="inlineStr"/>
       <c r="D109" t="inlineStr">
         <is>
-          <t>Naome Nshemereirwe</t>
+          <t>Nshemereirwe Naome</t>
         </is>
       </c>
     </row>
@@ -2396,7 +2396,7 @@
       <c r="C110" t="inlineStr"/>
       <c r="D110" t="inlineStr">
         <is>
-          <t>Ralph Munywevu</t>
+          <t>Munywevu Ralph</t>
         </is>
       </c>
     </row>
@@ -2414,7 +2414,7 @@
       <c r="C111" t="inlineStr"/>
       <c r="D111" t="inlineStr">
         <is>
-          <t>Asasira Azarius</t>
+          <t>Azarius Asasira</t>
         </is>
       </c>
     </row>
@@ -2432,7 +2432,7 @@
       <c r="C112" t="inlineStr"/>
       <c r="D112" t="inlineStr">
         <is>
-          <t>Solomon Amwesiga</t>
+          <t>Amwesiga Solomon</t>
         </is>
       </c>
     </row>
@@ -2450,7 +2450,7 @@
       <c r="C113" t="inlineStr"/>
       <c r="D113" t="inlineStr">
         <is>
-          <t>Remigious Tumwesigye</t>
+          <t>Tumwesigye Remigious</t>
         </is>
       </c>
     </row>
@@ -2468,7 +2468,7 @@
       <c r="C114" t="inlineStr"/>
       <c r="D114" t="inlineStr">
         <is>
-          <t>Lawrence Tumwebaze</t>
+          <t>Tumwebaze Lawrence</t>
         </is>
       </c>
     </row>
@@ -2486,7 +2486,7 @@
       <c r="C115" t="inlineStr"/>
       <c r="D115" t="inlineStr">
         <is>
-          <t>Doka Abdul</t>
+          <t>Abdul Doka</t>
         </is>
       </c>
     </row>
@@ -2504,7 +2504,7 @@
       <c r="C116" t="inlineStr"/>
       <c r="D116" t="inlineStr">
         <is>
-          <t>Sarah Kamuli</t>
+          <t>Kamuli Sarah</t>
         </is>
       </c>
     </row>
@@ -2522,7 +2522,7 @@
       <c r="C117" t="inlineStr"/>
       <c r="D117" t="inlineStr">
         <is>
-          <t>Inira Angucia</t>
+          <t>Angucia Inira</t>
         </is>
       </c>
     </row>
@@ -2540,7 +2540,7 @@
       <c r="C118" t="inlineStr"/>
       <c r="D118" t="inlineStr">
         <is>
-          <t>Gloria Acen</t>
+          <t>Acen Gloria</t>
         </is>
       </c>
     </row>
@@ -2558,7 +2558,7 @@
       <c r="C119" t="inlineStr"/>
       <c r="D119" t="inlineStr">
         <is>
-          <t>Geoffrey Mulinzi</t>
+          <t>Mulinzi Geoffrey</t>
         </is>
       </c>
     </row>
@@ -2576,7 +2576,7 @@
       <c r="C120" t="inlineStr"/>
       <c r="D120" t="inlineStr">
         <is>
-          <t>Erinah Zawedde</t>
+          <t>Zawedde Erinah</t>
         </is>
       </c>
     </row>
@@ -2594,7 +2594,7 @@
       <c r="C121" t="inlineStr"/>
       <c r="D121" t="inlineStr">
         <is>
-          <t>Christopher Odur</t>
+          <t>Odur Christopher</t>
         </is>
       </c>
     </row>
@@ -2612,7 +2612,7 @@
       <c r="C122" t="inlineStr"/>
       <c r="D122" t="inlineStr">
         <is>
-          <t>Harriet Ayikoru</t>
+          <t>Ayikoru Harriet</t>
         </is>
       </c>
     </row>
@@ -2630,7 +2630,7 @@
       <c r="C123" t="inlineStr"/>
       <c r="D123" t="inlineStr">
         <is>
-          <t>Atwine Andrew</t>
+          <t>Andrew Atwine</t>
         </is>
       </c>
     </row>
@@ -2648,7 +2648,7 @@
       <c r="C124" t="inlineStr"/>
       <c r="D124" t="inlineStr">
         <is>
-          <t>Stellah Rukundo</t>
+          <t>Rukundo Stellah</t>
         </is>
       </c>
     </row>
@@ -2666,7 +2666,7 @@
       <c r="C125" t="inlineStr"/>
       <c r="D125" t="inlineStr">
         <is>
-          <t>Alexander Opiru</t>
+          <t>Opiru Alexander</t>
         </is>
       </c>
     </row>
@@ -2684,7 +2684,7 @@
       <c r="C126" t="inlineStr"/>
       <c r="D126" t="inlineStr">
         <is>
-          <t>Godfrey Bogere</t>
+          <t>Bogere Godfrey</t>
         </is>
       </c>
     </row>
@@ -2702,7 +2702,7 @@
       <c r="C127" t="inlineStr"/>
       <c r="D127" t="inlineStr">
         <is>
-          <t>Joseline Kemigisa</t>
+          <t>Kemigisa Joseline</t>
         </is>
       </c>
     </row>
@@ -2720,7 +2720,7 @@
       <c r="C128" t="inlineStr"/>
       <c r="D128" t="inlineStr">
         <is>
-          <t>Jaliira Nakkazi</t>
+          <t>Nakkazi Jaliira</t>
         </is>
       </c>
     </row>
@@ -2738,7 +2738,7 @@
       <c r="C129" t="inlineStr"/>
       <c r="D129" t="inlineStr">
         <is>
-          <t>Kiiza Jude</t>
+          <t>Jude Kiiza</t>
         </is>
       </c>
     </row>
@@ -2756,7 +2756,7 @@
       <c r="C130" t="inlineStr"/>
       <c r="D130" t="inlineStr">
         <is>
-          <t>Bruce Ampaire</t>
+          <t>Ampaire Bruce</t>
         </is>
       </c>
     </row>
@@ -2774,7 +2774,7 @@
       <c r="C131" t="inlineStr"/>
       <c r="D131" t="inlineStr">
         <is>
-          <t>Alex Amoni</t>
+          <t>Amoni Alex</t>
         </is>
       </c>
     </row>
@@ -2792,7 +2792,7 @@
       <c r="C132" t="inlineStr"/>
       <c r="D132" t="inlineStr">
         <is>
-          <t>Nagaba Angel</t>
+          <t>Angel Nagaba</t>
         </is>
       </c>
     </row>
@@ -2810,7 +2810,7 @@
       <c r="C133" t="inlineStr"/>
       <c r="D133" t="inlineStr">
         <is>
-          <t>Mbabazi Grace</t>
+          <t>Grace Mbabazi</t>
         </is>
       </c>
     </row>
@@ -2828,7 +2828,7 @@
       <c r="C134" t="inlineStr"/>
       <c r="D134" t="inlineStr">
         <is>
-          <t>Muruubya Bruno</t>
+          <t>Bruno Muruubya</t>
         </is>
       </c>
     </row>
@@ -2846,7 +2846,7 @@
       <c r="C135" t="inlineStr"/>
       <c r="D135" t="inlineStr">
         <is>
-          <t>Stephen Okitoi</t>
+          <t>Okitoi Stephen</t>
         </is>
       </c>
     </row>
@@ -2864,7 +2864,7 @@
       <c r="C136" t="inlineStr"/>
       <c r="D136" t="inlineStr">
         <is>
-          <t>Kezekia Serwanga</t>
+          <t>Serwanga Kezekia</t>
         </is>
       </c>
     </row>
@@ -2882,7 +2882,7 @@
       <c r="C137" t="inlineStr"/>
       <c r="D137" t="inlineStr">
         <is>
-          <t>Margaret Orono</t>
+          <t>Orono Margaret</t>
         </is>
       </c>
     </row>
@@ -2900,7 +2900,7 @@
       <c r="C138" t="inlineStr"/>
       <c r="D138" t="inlineStr">
         <is>
-          <t>Joan Kizza</t>
+          <t>Kizza Joan</t>
         </is>
       </c>
     </row>
@@ -2918,7 +2918,7 @@
       <c r="C139" t="inlineStr"/>
       <c r="D139" t="inlineStr">
         <is>
-          <t>Rebecca Atenge</t>
+          <t>Atenge Rebecca</t>
         </is>
       </c>
     </row>
@@ -2936,7 +2936,7 @@
       <c r="C140" t="inlineStr"/>
       <c r="D140" t="inlineStr">
         <is>
-          <t>Rose Nakato</t>
+          <t>Nakato Rose</t>
         </is>
       </c>
     </row>
@@ -2954,7 +2954,7 @@
       <c r="C141" t="inlineStr"/>
       <c r="D141" t="inlineStr">
         <is>
-          <t>Madinah Nagujja</t>
+          <t>Nagujja Madinah</t>
         </is>
       </c>
     </row>
@@ -2972,7 +2972,7 @@
       <c r="C142" t="inlineStr"/>
       <c r="D142" t="inlineStr">
         <is>
-          <t>Gloria Suubi</t>
+          <t>Suubi Gloria</t>
         </is>
       </c>
     </row>
@@ -2990,7 +2990,7 @@
       <c r="C143" t="inlineStr"/>
       <c r="D143" t="inlineStr">
         <is>
-          <t>Stephen Olupot</t>
+          <t>Olupot Stephen</t>
         </is>
       </c>
     </row>
@@ -3008,7 +3008,7 @@
       <c r="C144" t="inlineStr"/>
       <c r="D144" t="inlineStr">
         <is>
-          <t>Sarah Namusubo</t>
+          <t>Namusubo Sarah</t>
         </is>
       </c>
     </row>
@@ -3026,7 +3026,7 @@
       <c r="C145" t="inlineStr"/>
       <c r="D145" t="inlineStr">
         <is>
-          <t>Marjorie Birabwa</t>
+          <t>Birabwa Marjorie</t>
         </is>
       </c>
     </row>
@@ -3044,7 +3044,7 @@
       <c r="C146" t="inlineStr"/>
       <c r="D146" t="inlineStr">
         <is>
-          <t>Ednah Asiimwe</t>
+          <t>Asiimwe Ednah</t>
         </is>
       </c>
     </row>
@@ -3062,7 +3062,7 @@
       <c r="C147" t="inlineStr"/>
       <c r="D147" t="inlineStr">
         <is>
-          <t>Silvano Alicabiaku</t>
+          <t>Alicabiaku Silvano</t>
         </is>
       </c>
     </row>
@@ -3080,7 +3080,7 @@
       <c r="C148" t="inlineStr"/>
       <c r="D148" t="inlineStr">
         <is>
-          <t>Betty Ituka</t>
+          <t>Ituka Betty</t>
         </is>
       </c>
     </row>
@@ -3098,7 +3098,7 @@
       <c r="C149" t="inlineStr"/>
       <c r="D149" t="inlineStr">
         <is>
-          <t>Eva Namukoli</t>
+          <t>Namukoli Eva</t>
         </is>
       </c>
     </row>
@@ -3116,7 +3116,7 @@
       <c r="C150" t="inlineStr"/>
       <c r="D150" t="inlineStr">
         <is>
-          <t>Jackline Nabaasa</t>
+          <t>Nabaasa Jackline</t>
         </is>
       </c>
     </row>
@@ -3134,7 +3134,7 @@
       <c r="C151" t="inlineStr"/>
       <c r="D151" t="inlineStr">
         <is>
-          <t>Priscilla Nankya</t>
+          <t>Nankya Priscilla</t>
         </is>
       </c>
     </row>
@@ -3152,7 +3152,7 @@
       <c r="C152" t="inlineStr"/>
       <c r="D152" t="inlineStr">
         <is>
-          <t>Samalie Nankya</t>
+          <t>Nankya Samalie</t>
         </is>
       </c>
     </row>
@@ -3170,7 +3170,7 @@
       <c r="C153" t="inlineStr"/>
       <c r="D153" t="inlineStr">
         <is>
-          <t>Martha Asinai</t>
+          <t>Asinai Martha</t>
         </is>
       </c>
     </row>
@@ -3188,7 +3188,7 @@
       <c r="C154" t="inlineStr"/>
       <c r="D154" t="inlineStr">
         <is>
-          <t>Kirabo Luzinda</t>
+          <t>Luzinda Kirabo</t>
         </is>
       </c>
     </row>
@@ -3206,7 +3206,7 @@
       <c r="C155" t="inlineStr"/>
       <c r="D155" t="inlineStr">
         <is>
-          <t>Irene Zawedde</t>
+          <t>Zawedde Irene</t>
         </is>
       </c>
     </row>
@@ -3224,7 +3224,7 @@
       <c r="C156" t="inlineStr"/>
       <c r="D156" t="inlineStr">
         <is>
-          <t>Angella Aloti</t>
+          <t>Aloti Angella</t>
         </is>
       </c>
     </row>
@@ -3242,7 +3242,7 @@
       <c r="C157" t="inlineStr"/>
       <c r="D157" t="inlineStr">
         <is>
-          <t>Honest Mpumwire</t>
+          <t>Mpumwire Honest</t>
         </is>
       </c>
     </row>
@@ -3260,7 +3260,7 @@
       <c r="C158" t="inlineStr"/>
       <c r="D158" t="inlineStr">
         <is>
-          <t>Shibbah Atuheire</t>
+          <t>Atuheire Shibbah</t>
         </is>
       </c>
     </row>
@@ -3278,7 +3278,7 @@
       <c r="C159" t="inlineStr"/>
       <c r="D159" t="inlineStr">
         <is>
-          <t>Wilson Langa</t>
+          <t>Langa Wilson</t>
         </is>
       </c>
     </row>
@@ -3296,7 +3296,7 @@
       <c r="C160" t="inlineStr"/>
       <c r="D160" t="inlineStr">
         <is>
-          <t>Doreen Akello</t>
+          <t>Akello Doreen</t>
         </is>
       </c>
     </row>
@@ -3314,7 +3314,7 @@
       <c r="C161" t="inlineStr"/>
       <c r="D161" t="inlineStr">
         <is>
-          <t>Mastulla Nalubega</t>
+          <t>Nalubega Mastulla</t>
         </is>
       </c>
     </row>
@@ -3332,7 +3332,7 @@
       <c r="C162" t="inlineStr"/>
       <c r="D162" t="inlineStr">
         <is>
-          <t>Lawrence Owomuhangi</t>
+          <t>Owomuhangi Lawrence</t>
         </is>
       </c>
     </row>
@@ -3350,7 +3350,7 @@
       <c r="C163" t="inlineStr"/>
       <c r="D163" t="inlineStr">
         <is>
-          <t>Victoria Kyohirwe</t>
+          <t>Kyohirwe Victoria</t>
         </is>
       </c>
     </row>
@@ -3368,7 +3368,7 @@
       <c r="C164" t="inlineStr"/>
       <c r="D164" t="inlineStr">
         <is>
-          <t>Patricia Komuhendo</t>
+          <t>Komuhendo Patricia</t>
         </is>
       </c>
     </row>
@@ -3386,7 +3386,7 @@
       <c r="C165" t="inlineStr"/>
       <c r="D165" t="inlineStr">
         <is>
-          <t>Ronald Aripa</t>
+          <t>Aripa Ronald</t>
         </is>
       </c>
     </row>
@@ -3404,7 +3404,7 @@
       <c r="C166" t="inlineStr"/>
       <c r="D166" t="inlineStr">
         <is>
-          <t>Johnson Mukunzi</t>
+          <t>Mukunzi Johnson</t>
         </is>
       </c>
     </row>
@@ -3422,7 +3422,7 @@
       <c r="C167" t="inlineStr"/>
       <c r="D167" t="inlineStr">
         <is>
-          <t>Clare Atuhaire</t>
+          <t>Atuhaire Clare</t>
         </is>
       </c>
     </row>
@@ -3440,7 +3440,7 @@
       <c r="C168" t="inlineStr"/>
       <c r="D168" t="inlineStr">
         <is>
-          <t>Denis Muhoozi</t>
+          <t>Muhoozi Denis</t>
         </is>
       </c>
     </row>
@@ -3458,7 +3458,7 @@
       <c r="C169" t="inlineStr"/>
       <c r="D169" t="inlineStr">
         <is>
-          <t>Bridget Kalanguka</t>
+          <t>Kalanguka Bridget</t>
         </is>
       </c>
     </row>
@@ -3476,7 +3476,7 @@
       <c r="C170" t="inlineStr"/>
       <c r="D170" t="inlineStr">
         <is>
-          <t>Sheba Kagwisa</t>
+          <t>Kagwisa Sheba</t>
         </is>
       </c>
     </row>
@@ -3494,7 +3494,7 @@
       <c r="C171" t="inlineStr"/>
       <c r="D171" t="inlineStr">
         <is>
-          <t>Lydia Kisaakye</t>
+          <t>Kisaakye Lydia</t>
         </is>
       </c>
     </row>
@@ -3512,7 +3512,7 @@
       <c r="C172" t="inlineStr"/>
       <c r="D172" t="inlineStr">
         <is>
-          <t>Betty Naluyange</t>
+          <t>Naluyange Betty</t>
         </is>
       </c>
     </row>
@@ -3530,7 +3530,7 @@
       <c r="C173" t="inlineStr"/>
       <c r="D173" t="inlineStr">
         <is>
-          <t>Kadaali Mudondo</t>
+          <t>Mudondo Kadaali</t>
         </is>
       </c>
     </row>
@@ -3548,7 +3548,7 @@
       <c r="C174" t="inlineStr"/>
       <c r="D174" t="inlineStr">
         <is>
-          <t>Aisha Nanteza</t>
+          <t>Nanteza Aisha</t>
         </is>
       </c>
     </row>
@@ -3566,7 +3566,7 @@
       <c r="C175" t="inlineStr"/>
       <c r="D175" t="inlineStr">
         <is>
-          <t>Doreen Namwima</t>
+          <t>Namwima Doreen</t>
         </is>
       </c>
     </row>
@@ -3584,7 +3584,7 @@
       <c r="C176" t="inlineStr"/>
       <c r="D176" t="inlineStr">
         <is>
-          <t>Kalanda Aaron</t>
+          <t>Aaron Kalanda</t>
         </is>
       </c>
     </row>
@@ -3602,7 +3602,7 @@
       <c r="C177" t="inlineStr"/>
       <c r="D177" t="inlineStr">
         <is>
-          <t>Christine Nabulime</t>
+          <t>Nabulime Christine</t>
         </is>
       </c>
     </row>
@@ -3620,7 +3620,7 @@
       <c r="C178" t="inlineStr"/>
       <c r="D178" t="inlineStr">
         <is>
-          <t>Christine Busingye</t>
+          <t>Busingye Christine</t>
         </is>
       </c>
     </row>
@@ -3638,7 +3638,7 @@
       <c r="C179" t="inlineStr"/>
       <c r="D179" t="inlineStr">
         <is>
-          <t>Fiona Namara</t>
+          <t>Namara Fiona</t>
         </is>
       </c>
     </row>
@@ -3656,7 +3656,7 @@
       <c r="C180" t="inlineStr"/>
       <c r="D180" t="inlineStr">
         <is>
-          <t>Roselyne Natukunda</t>
+          <t>Natukunda Roselyne</t>
         </is>
       </c>
     </row>
@@ -3674,7 +3674,7 @@
       <c r="C181" t="inlineStr"/>
       <c r="D181" t="inlineStr">
         <is>
-          <t>Michael Lubega</t>
+          <t>Lubega Michael</t>
         </is>
       </c>
     </row>
@@ -3692,7 +3692,7 @@
       <c r="C182" t="inlineStr"/>
       <c r="D182" t="inlineStr">
         <is>
-          <t>Christine Ainembabazi</t>
+          <t>Ainembabazi Christine</t>
         </is>
       </c>
     </row>
@@ -3710,7 +3710,7 @@
       <c r="C183" t="inlineStr"/>
       <c r="D183" t="inlineStr">
         <is>
-          <t>Norah Nansamba</t>
+          <t>Nansamba Norah</t>
         </is>
       </c>
     </row>
@@ -3728,7 +3728,7 @@
       <c r="C184" t="inlineStr"/>
       <c r="D184" t="inlineStr">
         <is>
-          <t>Lillian Onyait</t>
+          <t>Onyait Lillian</t>
         </is>
       </c>
     </row>
@@ -3746,7 +3746,7 @@
       <c r="C185" t="inlineStr"/>
       <c r="D185" t="inlineStr">
         <is>
-          <t>Musoke Alemu</t>
+          <t>Alemu Musoke</t>
         </is>
       </c>
     </row>
@@ -3764,7 +3764,7 @@
       <c r="C186" t="inlineStr"/>
       <c r="D186" t="inlineStr">
         <is>
-          <t>Paul Sawula</t>
+          <t>Sawula Paul</t>
         </is>
       </c>
     </row>
@@ -3782,7 +3782,7 @@
       <c r="C187" t="inlineStr"/>
       <c r="D187" t="inlineStr">
         <is>
-          <t>Esther Mbabazi</t>
+          <t>Mbabazi Esther</t>
         </is>
       </c>
     </row>
@@ -3800,7 +3800,7 @@
       <c r="C188" t="inlineStr"/>
       <c r="D188" t="inlineStr">
         <is>
-          <t>Primerose Nabaasa</t>
+          <t>Nabaasa Primerose</t>
         </is>
       </c>
     </row>
@@ -3818,7 +3818,7 @@
       <c r="C189" t="inlineStr"/>
       <c r="D189" t="inlineStr">
         <is>
-          <t>Benon Sembatya</t>
+          <t>Sembatya Benon</t>
         </is>
       </c>
     </row>
@@ -3836,7 +3836,7 @@
       <c r="C190" t="inlineStr"/>
       <c r="D190" t="inlineStr">
         <is>
-          <t>Peter Ssenkungu</t>
+          <t>Ssenkungu Peter</t>
         </is>
       </c>
     </row>
@@ -3854,7 +3854,7 @@
       <c r="C191" t="inlineStr"/>
       <c r="D191" t="inlineStr">
         <is>
-          <t>Alphonsina Wahumura</t>
+          <t>Wahumura Alphonsina</t>
         </is>
       </c>
     </row>
@@ -3872,7 +3872,7 @@
       <c r="C192" t="inlineStr"/>
       <c r="D192" t="inlineStr">
         <is>
-          <t>Nalubowa Olivia</t>
+          <t>Olivia Nalubowa</t>
         </is>
       </c>
     </row>
@@ -3890,7 +3890,7 @@
       <c r="C193" t="inlineStr"/>
       <c r="D193" t="inlineStr">
         <is>
-          <t>Gloria Nakiyemba</t>
+          <t>Nakiyemba Gloria</t>
         </is>
       </c>
     </row>
@@ -3908,7 +3908,7 @@
       <c r="C194" t="inlineStr"/>
       <c r="D194" t="inlineStr">
         <is>
-          <t>Barbara Nakiwala</t>
+          <t>Nakiwala Barbara</t>
         </is>
       </c>
     </row>
@@ -3926,7 +3926,7 @@
       <c r="C195" t="inlineStr"/>
       <c r="D195" t="inlineStr">
         <is>
-          <t>Paul Mpalaganyi</t>
+          <t>Mpalaganyi Paul</t>
         </is>
       </c>
     </row>
@@ -3944,7 +3944,7 @@
       <c r="C196" t="inlineStr"/>
       <c r="D196" t="inlineStr">
         <is>
-          <t>Lunkuse Kakumba</t>
+          <t>Kakumba Lunkuse</t>
         </is>
       </c>
     </row>
@@ -3962,7 +3962,7 @@
       <c r="C197" t="inlineStr"/>
       <c r="D197" t="inlineStr">
         <is>
-          <t>Naome Nansamba</t>
+          <t>Nansamba Naome</t>
         </is>
       </c>
     </row>
@@ -3980,7 +3980,7 @@
       <c r="C198" t="inlineStr"/>
       <c r="D198" t="inlineStr">
         <is>
-          <t>Fred Kasajja</t>
+          <t>Kasajja Fred</t>
         </is>
       </c>
     </row>
@@ -3998,7 +3998,7 @@
       <c r="C199" t="inlineStr"/>
       <c r="D199" t="inlineStr">
         <is>
-          <t>Andrew Mulondo</t>
+          <t>Mulondo Andrew</t>
         </is>
       </c>
     </row>
@@ -4016,7 +4016,7 @@
       <c r="C200" t="inlineStr"/>
       <c r="D200" t="inlineStr">
         <is>
-          <t>Javilla Ayebare</t>
+          <t>Ayebare Javilla</t>
         </is>
       </c>
     </row>
@@ -4034,7 +4034,7 @@
       <c r="C201" t="inlineStr"/>
       <c r="D201" t="inlineStr">
         <is>
-          <t>Anna Maria Sanyu</t>
+          <t>Sanyu Maria</t>
         </is>
       </c>
     </row>
@@ -4052,7 +4052,7 @@
       <c r="C202" t="inlineStr"/>
       <c r="D202" t="inlineStr">
         <is>
-          <t>Patience Charity</t>
+          <t>Charity Patience</t>
         </is>
       </c>
     </row>
@@ -4070,7 +4070,7 @@
       <c r="C203" t="inlineStr"/>
       <c r="D203" t="inlineStr">
         <is>
-          <t>Buwembo Musaazi</t>
+          <t>Musaazi Buwembo</t>
         </is>
       </c>
     </row>
@@ -4088,7 +4088,7 @@
       <c r="C204" t="inlineStr"/>
       <c r="D204" t="inlineStr">
         <is>
-          <t>Ruth Kyomuhendo</t>
+          <t>Kyomuhendo Ruth</t>
         </is>
       </c>
     </row>
@@ -4106,7 +4106,7 @@
       <c r="C205" t="inlineStr"/>
       <c r="D205" t="inlineStr">
         <is>
-          <t>Mary Babita</t>
+          <t>Babita Mary</t>
         </is>
       </c>
     </row>
@@ -4124,7 +4124,7 @@
       <c r="C206" t="inlineStr"/>
       <c r="D206" t="inlineStr">
         <is>
-          <t>Vicky Namutosi</t>
+          <t>Namutosi Vicky</t>
         </is>
       </c>
     </row>
@@ -4142,7 +4142,7 @@
       <c r="C207" t="inlineStr"/>
       <c r="D207" t="inlineStr">
         <is>
-          <t>Christine Babirye</t>
+          <t>Babirye Christine</t>
         </is>
       </c>
     </row>
@@ -4160,7 +4160,7 @@
       <c r="C208" t="inlineStr"/>
       <c r="D208" t="inlineStr">
         <is>
-          <t>Pearl Owomugisha</t>
+          <t>Owomugisha Pearl</t>
         </is>
       </c>
     </row>
@@ -4178,7 +4178,7 @@
       <c r="C209" t="inlineStr"/>
       <c r="D209" t="inlineStr">
         <is>
-          <t>Grace Nakaziba</t>
+          <t>Nakaziba Grace</t>
         </is>
       </c>
     </row>
@@ -4196,7 +4196,7 @@
       <c r="C210" t="inlineStr"/>
       <c r="D210" t="inlineStr">
         <is>
-          <t>Christine Akurut</t>
+          <t>Akurut Christine</t>
         </is>
       </c>
     </row>
@@ -4214,7 +4214,7 @@
       <c r="C211" t="inlineStr"/>
       <c r="D211" t="inlineStr">
         <is>
-          <t>Monica Muwanse</t>
+          <t>Muwanse Monica</t>
         </is>
       </c>
     </row>
@@ -4232,7 +4232,7 @@
       <c r="C212" t="inlineStr"/>
       <c r="D212" t="inlineStr">
         <is>
-          <t>Jackie Namatovu</t>
+          <t>Namatovu Jackie</t>
         </is>
       </c>
     </row>
@@ -4250,7 +4250,7 @@
       <c r="C213" t="inlineStr"/>
       <c r="D213" t="inlineStr">
         <is>
-          <t>Bernadette Ssemakula</t>
+          <t>Ssemakula Bernadette</t>
         </is>
       </c>
     </row>
@@ -4268,7 +4268,7 @@
       <c r="C214" t="inlineStr"/>
       <c r="D214" t="inlineStr">
         <is>
-          <t>Osbert Asiimwe</t>
+          <t>Asiimwe Osbert</t>
         </is>
       </c>
     </row>
@@ -4286,7 +4286,7 @@
       <c r="C215" t="inlineStr"/>
       <c r="D215" t="inlineStr">
         <is>
-          <t>Kenneth Akimanzi</t>
+          <t>Akimanzi Kenneth</t>
         </is>
       </c>
     </row>
@@ -4304,7 +4304,7 @@
       <c r="C216" t="inlineStr"/>
       <c r="D216" t="inlineStr">
         <is>
-          <t>Nyesigire Nagadya</t>
+          <t>Nagadya Nyesigire</t>
         </is>
       </c>
     </row>
@@ -4322,7 +4322,7 @@
       <c r="C217" t="inlineStr"/>
       <c r="D217" t="inlineStr">
         <is>
-          <t>Waiswa Sajjabi</t>
+          <t>Sajjabi Waiswa</t>
         </is>
       </c>
     </row>
@@ -4340,7 +4340,7 @@
       <c r="C218" t="inlineStr"/>
       <c r="D218" t="inlineStr">
         <is>
-          <t>Otim Jorem</t>
+          <t>Jorem Otim</t>
         </is>
       </c>
     </row>
@@ -4358,7 +4358,7 @@
       <c r="C219" t="inlineStr"/>
       <c r="D219" t="inlineStr">
         <is>
-          <t>Robert Opiyo</t>
+          <t>Opiyo Robert</t>
         </is>
       </c>
     </row>
@@ -4376,7 +4376,7 @@
       <c r="C220" t="inlineStr"/>
       <c r="D220" t="inlineStr">
         <is>
-          <t>Kasundhe Fazira</t>
+          <t>Fazira Kasundhe</t>
         </is>
       </c>
     </row>
@@ -4394,7 +4394,7 @@
       <c r="C221" t="inlineStr"/>
       <c r="D221" t="inlineStr">
         <is>
-          <t>Hajirah Nabirye</t>
+          <t>Nabirye Hajirah</t>
         </is>
       </c>
     </row>
@@ -4412,7 +4412,7 @@
       <c r="C222" t="inlineStr"/>
       <c r="D222" t="inlineStr">
         <is>
-          <t>Stephen Waiswa</t>
+          <t>Waiswa Stephen</t>
         </is>
       </c>
     </row>
@@ -4430,7 +4430,7 @@
       <c r="C223" t="inlineStr"/>
       <c r="D223" t="inlineStr">
         <is>
-          <t>Charles Bagire</t>
+          <t>Bagire Charles</t>
         </is>
       </c>
     </row>
@@ -4448,7 +4448,7 @@
       <c r="C224" t="inlineStr"/>
       <c r="D224" t="inlineStr">
         <is>
-          <t>Din Ndifuna</t>
+          <t>Ndifuna Din</t>
         </is>
       </c>
     </row>
@@ -4466,7 +4466,7 @@
       <c r="C225" t="inlineStr"/>
       <c r="D225" t="inlineStr">
         <is>
-          <t>Molly Nabbosa</t>
+          <t>Nabbosa Molly</t>
         </is>
       </c>
     </row>
@@ -4484,7 +4484,7 @@
       <c r="C226" t="inlineStr"/>
       <c r="D226" t="inlineStr">
         <is>
-          <t>Davis Muhangi</t>
+          <t>Muhangi Davis</t>
         </is>
       </c>
     </row>
@@ -4502,7 +4502,7 @@
       <c r="C227" t="inlineStr"/>
       <c r="D227" t="inlineStr">
         <is>
-          <t>Nicholas Ongom</t>
+          <t>Ongom Nicholas</t>
         </is>
       </c>
     </row>
@@ -4520,7 +4520,7 @@
       <c r="C228" t="inlineStr"/>
       <c r="D228" t="inlineStr">
         <is>
-          <t>Joel Muganza</t>
+          <t>Muganza Joel</t>
         </is>
       </c>
     </row>
@@ -4538,7 +4538,7 @@
       <c r="C229" t="inlineStr"/>
       <c r="D229" t="inlineStr">
         <is>
-          <t>Robert Kanyonyi</t>
+          <t>Kanyonyi Robert</t>
         </is>
       </c>
     </row>
@@ -4556,7 +4556,7 @@
       <c r="C230" t="inlineStr"/>
       <c r="D230" t="inlineStr">
         <is>
-          <t>Wasswa Kizito</t>
+          <t>Kizito Wasswa</t>
         </is>
       </c>
     </row>
@@ -4574,7 +4574,7 @@
       <c r="C231" t="inlineStr"/>
       <c r="D231" t="inlineStr">
         <is>
-          <t>Robert Andama</t>
+          <t>Andama Robert</t>
         </is>
       </c>
     </row>
@@ -4592,7 +4592,7 @@
       <c r="C232" t="inlineStr"/>
       <c r="D232" t="inlineStr">
         <is>
-          <t>Oling Oryonga</t>
+          <t>Oryonga Oling</t>
         </is>
       </c>
     </row>
@@ -4610,7 +4610,7 @@
       <c r="C233" t="inlineStr"/>
       <c r="D233" t="inlineStr">
         <is>
-          <t>Moses Okirio</t>
+          <t>Okirio Moses</t>
         </is>
       </c>
     </row>
@@ -4628,7 +4628,7 @@
       <c r="C234" t="inlineStr"/>
       <c r="D234" t="inlineStr">
         <is>
-          <t>Elinah Namanya</t>
+          <t>Namanya Elinah</t>
         </is>
       </c>
     </row>
@@ -4646,7 +4646,7 @@
       <c r="C235" t="inlineStr"/>
       <c r="D235" t="inlineStr">
         <is>
-          <t>Emmanuel Arinaitwe</t>
+          <t>Arinaitwe Emmanuel</t>
         </is>
       </c>
     </row>
@@ -4664,7 +4664,7 @@
       <c r="C236" t="inlineStr"/>
       <c r="D236" t="inlineStr">
         <is>
-          <t>Herman Karugaba</t>
+          <t>Karugaba Herman</t>
         </is>
       </c>
     </row>
@@ -4682,7 +4682,7 @@
       <c r="C237" t="inlineStr"/>
       <c r="D237" t="inlineStr">
         <is>
-          <t>Patrick Atwijukire</t>
+          <t>Atwijukire Patrick</t>
         </is>
       </c>
     </row>
@@ -4700,7 +4700,7 @@
       <c r="C238" t="inlineStr"/>
       <c r="D238" t="inlineStr">
         <is>
-          <t>Barbara Aine-Amaani</t>
+          <t>Aine-Amaani Barbara</t>
         </is>
       </c>
     </row>
@@ -4718,7 +4718,7 @@
       <c r="C239" t="inlineStr"/>
       <c r="D239" t="inlineStr">
         <is>
-          <t>Hassan Kigundu</t>
+          <t>Kigundu Hassan</t>
         </is>
       </c>
     </row>
@@ -4736,7 +4736,7 @@
       <c r="C240" t="inlineStr"/>
       <c r="D240" t="inlineStr">
         <is>
-          <t>Moses Okiror</t>
+          <t>Okiror Moses</t>
         </is>
       </c>
     </row>
@@ -4754,7 +4754,7 @@
       <c r="C241" t="inlineStr"/>
       <c r="D241" t="inlineStr">
         <is>
-          <t>Patrick Eriu</t>
+          <t>Eriu Patrick</t>
         </is>
       </c>
     </row>
@@ -4772,7 +4772,7 @@
       <c r="C242" t="inlineStr"/>
       <c r="D242" t="inlineStr">
         <is>
-          <t>Timothy Opio</t>
+          <t>Opio Timothy</t>
         </is>
       </c>
     </row>
@@ -4790,7 +4790,7 @@
       <c r="C243" t="inlineStr"/>
       <c r="D243" t="inlineStr">
         <is>
-          <t>Michael Okiror</t>
+          <t>Okiror Michael</t>
         </is>
       </c>
     </row>
@@ -4808,7 +4808,7 @@
       <c r="C244" t="inlineStr"/>
       <c r="D244" t="inlineStr">
         <is>
-          <t>Humphrey Ogwang</t>
+          <t>Ogwang Humphrey</t>
         </is>
       </c>
     </row>
@@ -4826,7 +4826,7 @@
       <c r="C245" t="inlineStr"/>
       <c r="D245" t="inlineStr">
         <is>
-          <t>Ronald Luzzi</t>
+          <t>Luzzi Ronald</t>
         </is>
       </c>
     </row>
@@ -4844,7 +4844,7 @@
       <c r="C246" t="inlineStr"/>
       <c r="D246" t="inlineStr">
         <is>
-          <t>Sherry Komugisha</t>
+          <t>Komugisha Sherry</t>
         </is>
       </c>
     </row>
@@ -4862,7 +4862,7 @@
       <c r="C247" t="inlineStr"/>
       <c r="D247" t="inlineStr">
         <is>
-          <t>Leticia Ruth Amulen</t>
+          <t>Amulen Ruth</t>
         </is>
       </c>
     </row>
@@ -4880,7 +4880,7 @@
       <c r="C248" t="inlineStr"/>
       <c r="D248" t="inlineStr">
         <is>
-          <t>Warren Mwebaze</t>
+          <t>Mwebaze Warren</t>
         </is>
       </c>
     </row>
@@ -4898,7 +4898,7 @@
       <c r="C249" t="inlineStr"/>
       <c r="D249" t="inlineStr">
         <is>
-          <t>Denis Turyahabwe</t>
+          <t>Turyahabwe Denis</t>
         </is>
       </c>
     </row>
@@ -4916,7 +4916,7 @@
       <c r="C250" t="inlineStr"/>
       <c r="D250" t="inlineStr">
         <is>
-          <t>Tadeo Twahirwa</t>
+          <t>Twahirwa Tadeo</t>
         </is>
       </c>
     </row>
@@ -4934,7 +4934,7 @@
       <c r="C251" t="inlineStr"/>
       <c r="D251" t="inlineStr">
         <is>
-          <t>John Ecweu</t>
+          <t>Ecweu John</t>
         </is>
       </c>
     </row>
@@ -4952,7 +4952,7 @@
       <c r="C252" t="inlineStr"/>
       <c r="D252" t="inlineStr">
         <is>
-          <t>Seezi Nduhuura</t>
+          <t>Nduhuura Seezi</t>
         </is>
       </c>
     </row>
@@ -4970,7 +4970,7 @@
       <c r="C253" t="inlineStr"/>
       <c r="D253" t="inlineStr">
         <is>
-          <t>Joan Namaganda</t>
+          <t>Namaganda Joan</t>
         </is>
       </c>
     </row>
@@ -4988,7 +4988,7 @@
       <c r="C254" t="inlineStr"/>
       <c r="D254" t="inlineStr">
         <is>
-          <t>Robert Kairagura</t>
+          <t>Kairagura Robert</t>
         </is>
       </c>
     </row>
@@ -5006,7 +5006,7 @@
       <c r="C255" t="inlineStr"/>
       <c r="D255" t="inlineStr">
         <is>
-          <t>John Aheebwa</t>
+          <t>Aheebwa John</t>
         </is>
       </c>
     </row>
@@ -5024,7 +5024,7 @@
       <c r="C256" t="inlineStr"/>
       <c r="D256" t="inlineStr">
         <is>
-          <t>Selman Egonu</t>
+          <t>Egonu Selman</t>
         </is>
       </c>
     </row>
@@ -5042,7 +5042,7 @@
       <c r="C257" t="inlineStr"/>
       <c r="D257" t="inlineStr">
         <is>
-          <t>Ejiet Kassim</t>
+          <t>Kassim Ejiet</t>
         </is>
       </c>
     </row>
@@ -5060,7 +5060,7 @@
       <c r="C258" t="inlineStr"/>
       <c r="D258" t="inlineStr">
         <is>
-          <t>Sarah Nalule</t>
+          <t>Nalule Sarah</t>
         </is>
       </c>
     </row>
@@ -5078,7 +5078,7 @@
       <c r="C259" t="inlineStr"/>
       <c r="D259" t="inlineStr">
         <is>
-          <t>Rose Wegosasa</t>
+          <t>Wegosasa Rose</t>
         </is>
       </c>
     </row>
@@ -5096,7 +5096,7 @@
       <c r="C260" t="inlineStr"/>
       <c r="D260" t="inlineStr">
         <is>
-          <t>Christopher Wangi</t>
+          <t>Wangi Christopher</t>
         </is>
       </c>
     </row>
@@ -5114,7 +5114,7 @@
       <c r="C261" t="inlineStr"/>
       <c r="D261" t="inlineStr">
         <is>
-          <t>Gamisha Fatuma</t>
+          <t>Fatuma Gamisha</t>
         </is>
       </c>
     </row>
@@ -5132,7 +5132,7 @@
       <c r="C262" t="inlineStr"/>
       <c r="D262" t="inlineStr">
         <is>
-          <t>Ahmed Mayanja</t>
+          <t>Mayanja Ahmed</t>
         </is>
       </c>
     </row>
@@ -5150,7 +5150,7 @@
       <c r="C263" t="inlineStr"/>
       <c r="D263" t="inlineStr">
         <is>
-          <t>Drake Habiyaremye</t>
+          <t>Habiyaremye Drake</t>
         </is>
       </c>
     </row>
@@ -5168,7 +5168,7 @@
       <c r="C264" t="inlineStr"/>
       <c r="D264" t="inlineStr">
         <is>
-          <t>Arnest Bunkeddeko</t>
+          <t>Bunkeddeko Arnest</t>
         </is>
       </c>
     </row>
@@ -5186,7 +5186,7 @@
       <c r="C265" t="inlineStr"/>
       <c r="D265" t="inlineStr">
         <is>
-          <t>Vicky Kisembo</t>
+          <t>Kisembo Vicky</t>
         </is>
       </c>
     </row>
@@ -5204,7 +5204,7 @@
       <c r="C266" t="inlineStr"/>
       <c r="D266" t="inlineStr">
         <is>
-          <t>Moses Agaba</t>
+          <t>Agaba Moses</t>
         </is>
       </c>
     </row>
@@ -5222,7 +5222,7 @@
       <c r="C267" t="inlineStr"/>
       <c r="D267" t="inlineStr">
         <is>
-          <t>Anne Clare Nalunkuuma</t>
+          <t>Nalunkuuma Clare</t>
         </is>
       </c>
     </row>
@@ -5240,7 +5240,7 @@
       <c r="C268" t="inlineStr"/>
       <c r="D268" t="inlineStr">
         <is>
-          <t>Jenipher Nyiraguhirwa</t>
+          <t>Nyiraguhirwa Jenipher</t>
         </is>
       </c>
     </row>
@@ -5258,7 +5258,7 @@
       <c r="C269" t="inlineStr"/>
       <c r="D269" t="inlineStr">
         <is>
-          <t>Tonny Kirangwa</t>
+          <t>Kirangwa Tonny</t>
         </is>
       </c>
     </row>
@@ -5276,7 +5276,7 @@
       <c r="C270" t="inlineStr"/>
       <c r="D270" t="inlineStr">
         <is>
-          <t>Kanavita William</t>
+          <t>William Kanavita</t>
         </is>
       </c>
     </row>
@@ -5294,7 +5294,7 @@
       <c r="C271" t="inlineStr"/>
       <c r="D271" t="inlineStr">
         <is>
-          <t>Mary Musiimenta</t>
+          <t>Musiimenta Mary</t>
         </is>
       </c>
     </row>
@@ -5312,7 +5312,7 @@
       <c r="C272" t="inlineStr"/>
       <c r="D272" t="inlineStr">
         <is>
-          <t>Stuart Matsiko</t>
+          <t>Matsiko Stuart</t>
         </is>
       </c>
     </row>
@@ -5330,7 +5330,7 @@
       <c r="C273" t="inlineStr"/>
       <c r="D273" t="inlineStr">
         <is>
-          <t>Vallence Nkurunziza</t>
+          <t>Nkurunziza Vallence</t>
         </is>
       </c>
     </row>
@@ -5348,7 +5348,7 @@
       <c r="C274" t="inlineStr"/>
       <c r="D274" t="inlineStr">
         <is>
-          <t>Julian Ahabwe</t>
+          <t>Ahabwe Julian</t>
         </is>
       </c>
     </row>
@@ -5366,7 +5366,7 @@
       <c r="C275" t="inlineStr"/>
       <c r="D275" t="inlineStr">
         <is>
-          <t>Rwamatungi Mwesigwa</t>
+          <t>Mwesigwa Rwamatungi</t>
         </is>
       </c>
     </row>
@@ -5384,7 +5384,7 @@
       <c r="C276" t="inlineStr"/>
       <c r="D276" t="inlineStr">
         <is>
-          <t>Samuel Dadye</t>
+          <t>Dadye Samuel</t>
         </is>
       </c>
     </row>
@@ -5402,7 +5402,7 @@
       <c r="C277" t="inlineStr"/>
       <c r="D277" t="inlineStr">
         <is>
-          <t>Yusuf Kiiza</t>
+          <t>Kiiza Yusuf</t>
         </is>
       </c>
     </row>
@@ -5420,7 +5420,7 @@
       <c r="C278" t="inlineStr"/>
       <c r="D278" t="inlineStr">
         <is>
-          <t>Kajuma Irene</t>
+          <t>Irene Kajuma</t>
         </is>
       </c>
     </row>
@@ -5438,7 +5438,7 @@
       <c r="C279" t="inlineStr"/>
       <c r="D279" t="inlineStr">
         <is>
-          <t>Alfred Ocen</t>
+          <t>Ocen Alfred</t>
         </is>
       </c>
     </row>
@@ -5456,7 +5456,7 @@
       <c r="C280" t="inlineStr"/>
       <c r="D280" t="inlineStr">
         <is>
-          <t>Oliver Namaganda</t>
+          <t>Namaganda Oliver</t>
         </is>
       </c>
     </row>
@@ -5474,7 +5474,7 @@
       <c r="C281" t="inlineStr"/>
       <c r="D281" t="inlineStr">
         <is>
-          <t>Delany Otim</t>
+          <t>Otim Delany</t>
         </is>
       </c>
     </row>
@@ -5492,7 +5492,7 @@
       <c r="C282" t="inlineStr"/>
       <c r="D282" t="inlineStr">
         <is>
-          <t>Moses Mwesigye</t>
+          <t>Mwesigye Moses</t>
         </is>
       </c>
     </row>
@@ -5510,7 +5510,7 @@
       <c r="C283" t="inlineStr"/>
       <c r="D283" t="inlineStr">
         <is>
-          <t>Gordie Tugume</t>
+          <t>Tugume Gordie</t>
         </is>
       </c>
     </row>
@@ -5528,7 +5528,7 @@
       <c r="C284" t="inlineStr"/>
       <c r="D284" t="inlineStr">
         <is>
-          <t>Nivia Nangobi</t>
+          <t>Nangobi Nivia</t>
         </is>
       </c>
     </row>
@@ -5546,7 +5546,7 @@
       <c r="C285" t="inlineStr"/>
       <c r="D285" t="inlineStr">
         <is>
-          <t>George Mukoyonzo</t>
+          <t>Mukoyonzo George</t>
         </is>
       </c>
     </row>
@@ -5564,7 +5564,7 @@
       <c r="C286" t="inlineStr"/>
       <c r="D286" t="inlineStr">
         <is>
-          <t>Mathias Kalema</t>
+          <t>Kalema Mathias</t>
         </is>
       </c>
     </row>
@@ -5582,7 +5582,7 @@
       <c r="C287" t="inlineStr"/>
       <c r="D287" t="inlineStr">
         <is>
-          <t>Doreen Wandera</t>
+          <t>Wandera Doreen</t>
         </is>
       </c>
     </row>
@@ -5600,7 +5600,7 @@
       <c r="C288" t="inlineStr"/>
       <c r="D288" t="inlineStr">
         <is>
-          <t>Stephen Walangaire</t>
+          <t>Walangaire Stephen</t>
         </is>
       </c>
     </row>
@@ -5618,7 +5618,7 @@
       <c r="C289" t="inlineStr"/>
       <c r="D289" t="inlineStr">
         <is>
-          <t>Mulyagonja Winnie</t>
+          <t>Winnie Mulyagonja</t>
         </is>
       </c>
     </row>
@@ -5636,7 +5636,7 @@
       <c r="C290" t="inlineStr"/>
       <c r="D290" t="inlineStr">
         <is>
-          <t>Sandra Nabagereka</t>
+          <t>Nabagereka Sandra</t>
         </is>
       </c>
     </row>
@@ -5654,7 +5654,7 @@
       <c r="C291" t="inlineStr"/>
       <c r="D291" t="inlineStr">
         <is>
-          <t>Wasswa Paul</t>
+          <t>Paul Wasswa</t>
         </is>
       </c>
     </row>
@@ -5672,7 +5672,7 @@
       <c r="C292" t="inlineStr"/>
       <c r="D292" t="inlineStr">
         <is>
-          <t>Norah Atenia</t>
+          <t>Atenia Norah</t>
         </is>
       </c>
     </row>
@@ -5690,7 +5690,7 @@
       <c r="C293" t="inlineStr"/>
       <c r="D293" t="inlineStr">
         <is>
-          <t>Scovia Kobusinge</t>
+          <t>Kobusinge Scovia</t>
         </is>
       </c>
     </row>
@@ -5708,7 +5708,7 @@
       <c r="C294" t="inlineStr"/>
       <c r="D294" t="inlineStr">
         <is>
-          <t>Nuwagaba Doreen</t>
+          <t>Doreen Nuwagaba</t>
         </is>
       </c>
     </row>
@@ -5726,7 +5726,7 @@
       <c r="C295" t="inlineStr"/>
       <c r="D295" t="inlineStr">
         <is>
-          <t>Kasujja Irene</t>
+          <t>Irene Kasujja</t>
         </is>
       </c>
     </row>
@@ -5744,7 +5744,7 @@
       <c r="C296" t="inlineStr"/>
       <c r="D296" t="inlineStr">
         <is>
-          <t>Mbaziira Felix</t>
+          <t>Felix Mbaziira</t>
         </is>
       </c>
     </row>
@@ -5762,7 +5762,7 @@
       <c r="C297" t="inlineStr"/>
       <c r="D297" t="inlineStr">
         <is>
-          <t>Kebirungi Patricia</t>
+          <t>Patricia Kebirungi</t>
         </is>
       </c>
     </row>
@@ -5780,7 +5780,7 @@
       <c r="C298" t="inlineStr"/>
       <c r="D298" t="inlineStr">
         <is>
-          <t>Atugonza Winfred</t>
+          <t>Winfred Atugonza</t>
         </is>
       </c>
     </row>
@@ -5798,7 +5798,7 @@
       <c r="C299" t="inlineStr"/>
       <c r="D299" t="inlineStr">
         <is>
-          <t>Nalule Angella</t>
+          <t>Angella Nalule</t>
         </is>
       </c>
     </row>
@@ -5816,7 +5816,7 @@
       <c r="C300" t="inlineStr"/>
       <c r="D300" t="inlineStr">
         <is>
-          <t>Tusiimire Aderah</t>
+          <t>Aderah Tusiimire</t>
         </is>
       </c>
     </row>
@@ -5834,7 +5834,7 @@
       <c r="C301" t="inlineStr"/>
       <c r="D301" t="inlineStr">
         <is>
-          <t>Namale Sarah</t>
+          <t>Sarah Namale</t>
         </is>
       </c>
     </row>
@@ -5852,7 +5852,7 @@
       <c r="C302" t="inlineStr"/>
       <c r="D302" t="inlineStr">
         <is>
-          <t>Andrews Obbo</t>
+          <t>Obbo Andrews</t>
         </is>
       </c>
     </row>
@@ -5870,7 +5870,7 @@
       <c r="C303" t="inlineStr"/>
       <c r="D303" t="inlineStr">
         <is>
-          <t>Joanitor Aliisa</t>
+          <t>Aliisa Joanitor</t>
         </is>
       </c>
     </row>
@@ -5888,7 +5888,7 @@
       <c r="C304" t="inlineStr"/>
       <c r="D304" t="inlineStr">
         <is>
-          <t>Monicah Tugume</t>
+          <t>Tugume Monicah</t>
         </is>
       </c>
     </row>
@@ -5906,7 +5906,7 @@
       <c r="C305" t="inlineStr"/>
       <c r="D305" t="inlineStr">
         <is>
-          <t>Chrisostom Aharizira</t>
+          <t>Aharizira Chrisostom</t>
         </is>
       </c>
     </row>
@@ -5924,7 +5924,7 @@
       <c r="C306" t="inlineStr"/>
       <c r="D306" t="inlineStr">
         <is>
-          <t>Obadiah Kwikiriza</t>
+          <t>Kwikiriza Obadiah</t>
         </is>
       </c>
     </row>
@@ -5942,7 +5942,7 @@
       <c r="C307" t="inlineStr"/>
       <c r="D307" t="inlineStr">
         <is>
-          <t>Dorothy Natukunda</t>
+          <t>Natukunda Dorothy</t>
         </is>
       </c>
     </row>
@@ -5960,7 +5960,7 @@
       <c r="C308" t="inlineStr"/>
       <c r="D308" t="inlineStr">
         <is>
-          <t>Agnes Kyomuhendo</t>
+          <t>Kyomuhendo Agnes</t>
         </is>
       </c>
     </row>
@@ -5978,7 +5978,7 @@
       <c r="C309" t="inlineStr"/>
       <c r="D309" t="inlineStr">
         <is>
-          <t>Richard Muhigwa</t>
+          <t>Muhigwa Richard</t>
         </is>
       </c>
     </row>
@@ -5996,7 +5996,7 @@
       <c r="C310" t="inlineStr"/>
       <c r="D310" t="inlineStr">
         <is>
-          <t>Claire Naggayi</t>
+          <t>Naggayi Claire</t>
         </is>
       </c>
     </row>
@@ -6014,7 +6014,7 @@
       <c r="C311" t="inlineStr"/>
       <c r="D311" t="inlineStr">
         <is>
-          <t>Semanda Banenye Nalwoga</t>
+          <t>Nalwoga Banenye</t>
         </is>
       </c>
     </row>
@@ -6032,7 +6032,7 @@
       <c r="C312" t="inlineStr"/>
       <c r="D312" t="inlineStr">
         <is>
-          <t>Jacqueline Nalubega</t>
+          <t>Nalubega Jacqueline</t>
         </is>
       </c>
     </row>
@@ -6050,7 +6050,7 @@
       <c r="C313" t="inlineStr"/>
       <c r="D313" t="inlineStr">
         <is>
-          <t>Jemimah Akedi</t>
+          <t>Akedi Jemimah</t>
         </is>
       </c>
     </row>
@@ -6068,7 +6068,7 @@
       <c r="C314" t="inlineStr"/>
       <c r="D314" t="inlineStr">
         <is>
-          <t>Flavia Namirimu</t>
+          <t>Namirimu Flavia</t>
         </is>
       </c>
     </row>
@@ -6086,7 +6086,7 @@
       <c r="C315" t="inlineStr"/>
       <c r="D315" t="inlineStr">
         <is>
-          <t>Doreen Ankunda</t>
+          <t>Ankunda Doreen</t>
         </is>
       </c>
     </row>
@@ -6104,7 +6104,7 @@
       <c r="C316" t="inlineStr"/>
       <c r="D316" t="inlineStr">
         <is>
-          <t>Muhammed Abdulhakim</t>
+          <t>Abdulhakim Muhammed</t>
         </is>
       </c>
     </row>
@@ -6122,7 +6122,7 @@
       <c r="C317" t="inlineStr"/>
       <c r="D317" t="inlineStr">
         <is>
-          <t>Oscar Omona</t>
+          <t>Omona Oscar</t>
         </is>
       </c>
     </row>
@@ -6140,7 +6140,7 @@
       <c r="C318" t="inlineStr"/>
       <c r="D318" t="inlineStr">
         <is>
-          <t>Lugemwa Mukasa Gonzaga</t>
+          <t>Gonzaga Mukasa</t>
         </is>
       </c>
     </row>
@@ -6158,7 +6158,7 @@
       <c r="C319" t="inlineStr"/>
       <c r="D319" t="inlineStr">
         <is>
-          <t>Komugisa Hilda</t>
+          <t>Hilda Komugisa</t>
         </is>
       </c>
     </row>
@@ -6176,7 +6176,7 @@
       <c r="C320" t="inlineStr"/>
       <c r="D320" t="inlineStr">
         <is>
-          <t>Auma Santina</t>
+          <t>Santina Auma</t>
         </is>
       </c>
     </row>
@@ -6194,7 +6194,7 @@
       <c r="C321" t="inlineStr"/>
       <c r="D321" t="inlineStr">
         <is>
-          <t>Patrick Achou</t>
+          <t>Achou Patrick</t>
         </is>
       </c>
     </row>
@@ -6212,7 +6212,7 @@
       <c r="C322" t="inlineStr"/>
       <c r="D322" t="inlineStr">
         <is>
-          <t>Sera Nerima</t>
+          <t>Nerima Sera</t>
         </is>
       </c>
     </row>
@@ -6230,7 +6230,7 @@
       <c r="C323" t="inlineStr"/>
       <c r="D323" t="inlineStr">
         <is>
-          <t>Alex Alemukori</t>
+          <t>Alemukori Alex</t>
         </is>
       </c>
     </row>
@@ -6248,7 +6248,7 @@
       <c r="C324" t="inlineStr"/>
       <c r="D324" t="inlineStr">
         <is>
-          <t>Daniel Ojoo</t>
+          <t>Ojoo Daniel</t>
         </is>
       </c>
     </row>
@@ -6266,7 +6266,7 @@
       <c r="C325" t="inlineStr"/>
       <c r="D325" t="inlineStr">
         <is>
-          <t>Anitah Nagujja</t>
+          <t>Nagujja Anitah</t>
         </is>
       </c>
     </row>
@@ -6284,7 +6284,7 @@
       <c r="C326" t="inlineStr"/>
       <c r="D326" t="inlineStr">
         <is>
-          <t>Abraham Imuaan</t>
+          <t>Imuaan Abraham</t>
         </is>
       </c>
     </row>
@@ -6302,7 +6302,7 @@
       <c r="C327" t="inlineStr"/>
       <c r="D327" t="inlineStr">
         <is>
-          <t>Mabonga Geofrey</t>
+          <t>Geofrey Mabonga</t>
         </is>
       </c>
     </row>
@@ -6320,7 +6320,7 @@
       <c r="C328" t="inlineStr"/>
       <c r="D328" t="inlineStr">
         <is>
-          <t>Angella Nyakecho</t>
+          <t>Nyakecho Angella</t>
         </is>
       </c>
     </row>
@@ -6338,7 +6338,7 @@
       <c r="C329" t="inlineStr"/>
       <c r="D329" t="inlineStr">
         <is>
-          <t>Mugwanya Deus O Kasirye</t>
+          <t>Kasirye O</t>
         </is>
       </c>
     </row>
@@ -6356,7 +6356,7 @@
       <c r="C330" t="inlineStr"/>
       <c r="D330" t="inlineStr">
         <is>
-          <t>Owori Amanda</t>
+          <t>Amanda Owori</t>
         </is>
       </c>
     </row>
@@ -6374,7 +6374,7 @@
       <c r="C331" t="inlineStr"/>
       <c r="D331" t="inlineStr">
         <is>
-          <t>Godwin Rwanyaga</t>
+          <t>Rwanyaga Godwin</t>
         </is>
       </c>
     </row>
@@ -6392,7 +6392,7 @@
       <c r="C332" t="inlineStr"/>
       <c r="D332" t="inlineStr">
         <is>
-          <t>Gloria Kharono</t>
+          <t>Kharono Gloria</t>
         </is>
       </c>
     </row>
@@ -6410,7 +6410,7 @@
       <c r="C333" t="inlineStr"/>
       <c r="D333" t="inlineStr">
         <is>
-          <t>Peter Byamukama</t>
+          <t>Byamukama Peter</t>
         </is>
       </c>
     </row>
@@ -6428,7 +6428,7 @@
       <c r="C334" t="inlineStr"/>
       <c r="D334" t="inlineStr">
         <is>
-          <t>Claire Ichumar</t>
+          <t>Ichumar Claire</t>
         </is>
       </c>
     </row>
@@ -6446,7 +6446,7 @@
       <c r="C335" t="inlineStr"/>
       <c r="D335" t="inlineStr">
         <is>
-          <t>Teopista Nakigudde</t>
+          <t>Nakigudde Teopista</t>
         </is>
       </c>
     </row>
@@ -6464,7 +6464,7 @@
       <c r="C336" t="inlineStr"/>
       <c r="D336" t="inlineStr">
         <is>
-          <t>Lillian Komugisha</t>
+          <t>Komugisha Lillian</t>
         </is>
       </c>
     </row>
@@ -6482,7 +6482,7 @@
       <c r="C337" t="inlineStr"/>
       <c r="D337" t="inlineStr">
         <is>
-          <t>Nakiranda Sajjabi</t>
+          <t>Sajjabi Nakiranda</t>
         </is>
       </c>
     </row>
@@ -6500,7 +6500,7 @@
       <c r="C338" t="inlineStr"/>
       <c r="D338" t="inlineStr">
         <is>
-          <t>Najia Namayanja</t>
+          <t>Namayanja Najia</t>
         </is>
       </c>
     </row>
@@ -6518,7 +6518,7 @@
       <c r="C339" t="inlineStr"/>
       <c r="D339" t="inlineStr">
         <is>
-          <t>Simon Wanyama</t>
+          <t>Wanyama Simon</t>
         </is>
       </c>
     </row>
@@ -6536,7 +6536,7 @@
       <c r="C340" t="inlineStr"/>
       <c r="D340" t="inlineStr">
         <is>
-          <t>Brenda Muyinza</t>
+          <t>Muyinza Brenda</t>
         </is>
       </c>
     </row>
@@ -6554,7 +6554,7 @@
       <c r="C341" t="inlineStr"/>
       <c r="D341" t="inlineStr">
         <is>
-          <t>Nakandi Kakyama</t>
+          <t>Kakyama Nakandi</t>
         </is>
       </c>
     </row>
@@ -6572,7 +6572,7 @@
       <c r="C342" t="inlineStr"/>
       <c r="D342" t="inlineStr">
         <is>
-          <t>Atukunda Shallot</t>
+          <t>Shallot Atukunda</t>
         </is>
       </c>
     </row>
@@ -6590,7 +6590,7 @@
       <c r="C343" t="inlineStr"/>
       <c r="D343" t="inlineStr">
         <is>
-          <t>Grace Ileka</t>
+          <t>Ileka Grace</t>
         </is>
       </c>
     </row>
@@ -6608,7 +6608,7 @@
       <c r="C344" t="inlineStr"/>
       <c r="D344" t="inlineStr">
         <is>
-          <t>Joseph Emuria</t>
+          <t>Emuria Joseph</t>
         </is>
       </c>
     </row>
@@ -6626,7 +6626,7 @@
       <c r="C345" t="inlineStr"/>
       <c r="D345" t="inlineStr">
         <is>
-          <t>Michael Mugisa</t>
+          <t>Mugisa Michael</t>
         </is>
       </c>
     </row>
@@ -6644,7 +6644,7 @@
       <c r="C346" t="inlineStr"/>
       <c r="D346" t="inlineStr">
         <is>
-          <t>Peterson Atuhairwe</t>
+          <t>Atuhairwe Peterson</t>
         </is>
       </c>
     </row>

</xml_diff>